<commit_message>
sotos-produce-market: 20 articles per month
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/sotos-produce-market/keyword-research.xlsx
+++ b/decks/sotos-produce-market/keyword-research.xlsx
@@ -1744,12 +1744,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Month 2</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Best current target</t>
+          <t>Month 1</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Near-final</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -1759,28 +1759,28 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Fundraising Ideas for Sports Teams, Sorted by Effort and Payoff</t>
+          <t>Winter Fundraising Ideas for January and February</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>fundraising ideas for sports teams</t>
+          <t>winter fundraising ideas</t>
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>1300</v>
+        <v>260</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>Very Easy</t>
         </is>
       </c>
-      <c r="J21" s="13" t="inlineStr">
-        <is>
-          <t>Fundraisers for Sports Teams</t>
+      <c r="J21" s="12" t="inlineStr">
+        <is>
+          <t>School, Church and Club Fundraisers</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="L21" s="7" t="inlineStr">
         <is>
-          <t>Also covers: sports fundraising ideas, fundraisers for sports teams, sports fundraisers, good fundraisers for sports teams, best fundraisers for sports teams, most profitable fundraisers for sports teams, best team fundraisers, best fundraising ideas for sports teams and 18 more.</t>
+          <t>Seasonal: published in month 1 so it has time to rank before January. Also covers: winter fundraising ideas schools.</t>
         </is>
       </c>
     </row>
@@ -1815,23 +1815,23 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Youth Sports Fundraising Ideas Parents Can Run on a Weekend</t>
+          <t>Fundraising Ideas for Sports Teams, Sorted by Effort and Payoff</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>youth sports fundraising ideas</t>
+          <t>fundraising ideas for sports teams</t>
         </is>
       </c>
       <c r="G22" s="4" t="n">
-        <v>320</v>
-      </c>
-      <c r="H22" s="9" t="n">
-        <v>16</v>
+        <v>1300</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>11</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="J22" s="13" t="inlineStr">
@@ -1846,7 +1846,7 @@
       </c>
       <c r="L22" s="7" t="inlineStr">
         <is>
-          <t>Also covers: fundraising ideas for youth sports teams, money raising ideas for sports clubs, fundraising ideas for sports clubs.</t>
+          <t>Also covers: sports fundraising ideas, fundraisers for sports teams, sports fundraisers, good fundraisers for sports teams, best fundraisers for sports teams, most profitable fundraisers for sports teams, best team fundraisers, best fundraising ideas for sports teams and 18 more.</t>
         </is>
       </c>
     </row>
@@ -1871,23 +1871,23 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Baseball Fundraising Ideas That Fit Around Practice and Game Days</t>
+          <t>Youth Sports Fundraising Ideas Parents Can Run on a Weekend</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>baseball fundraising ideas</t>
+          <t>youth sports fundraising ideas</t>
         </is>
       </c>
       <c r="G23" s="4" t="n">
-        <v>590</v>
-      </c>
-      <c r="H23" s="5" t="n">
-        <v>8</v>
+        <v>320</v>
+      </c>
+      <c r="H23" s="9" t="n">
+        <v>16</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Very Easy</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="J23" s="13" t="inlineStr">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="L23" s="7" t="inlineStr">
         <is>
-          <t>Also covers: baseball team fundraising ideas, baseball fundraiser, baseball team fundraiser.</t>
+          <t>Also covers: fundraising ideas for youth sports teams, money raising ideas for sports clubs, fundraising ideas for sports clubs.</t>
         </is>
       </c>
     </row>
@@ -1927,19 +1927,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Basketball Fundraiser Ideas Built Around Home Games and Tournaments</t>
+          <t>Baseball Fundraising Ideas That Fit Around Practice and Game Days</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>basketball fundraiser</t>
+          <t>baseball fundraising ideas</t>
         </is>
       </c>
       <c r="G24" s="4" t="n">
-        <v>480</v>
+        <v>590</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1958,7 +1958,7 @@
       </c>
       <c r="L24" s="7" t="inlineStr">
         <is>
-          <t>Also covers: basketball fundraising ideas, fundraising ideas for basketball team, the perfect basketball fundraiser, fundraising for basketball teams, high school basketball fundraising ideas, aau basketball fundraising ideas.</t>
+          <t>Also covers: baseball team fundraising ideas, baseball fundraiser, baseball team fundraiser.</t>
         </is>
       </c>
     </row>
@@ -1983,19 +1983,19 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Football Fundraising Ideas to Cover Gear and Away Games</t>
+          <t>Basketball Fundraiser Ideas Built Around Home Games and Tournaments</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>football fundraising ideas</t>
+          <t>basketball fundraiser</t>
         </is>
       </c>
       <c r="G25" s="4" t="n">
         <v>480</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="L25" s="7" t="inlineStr">
         <is>
-          <t>Also covers: football fundraiser, fundraising ideas for football teams, high school football fundraising ideas, fundraising for football teams, fundraising ideas for youth football, exciting youth football fundraising ideas, fundraising ideas for football clubs, football field fundraiser.</t>
+          <t>Also covers: basketball fundraising ideas, fundraising ideas for basketball team, the perfect basketball fundraiser, fundraising for basketball teams, high school basketball fundraising ideas, aau basketball fundraising ideas.</t>
         </is>
       </c>
     </row>
@@ -2039,19 +2039,19 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Fundraising for Soccer Teams Facing Club and Tournament Fees</t>
+          <t>Football Fundraising Ideas to Cover Gear and Away Games</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>fundraising for soccer teams</t>
+          <t>football fundraising ideas</t>
         </is>
       </c>
       <c r="G26" s="4" t="n">
-        <v>140</v>
+        <v>480</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="L26" s="7" t="inlineStr">
         <is>
-          <t>Also covers: fundraising ideas for soccer clubs.</t>
+          <t>Also covers: football fundraiser, fundraising ideas for football teams, high school football fundraising ideas, fundraising for football teams, fundraising ideas for youth football, exciting youth football fundraising ideas, fundraising ideas for football clubs, football field fundraiser.</t>
         </is>
       </c>
     </row>
@@ -2095,16 +2095,16 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Track and Field Fundraising Ideas for Meet Season and Cross Country</t>
+          <t>Fundraising for Soccer Teams Facing Club and Tournament Fees</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>track and field fundraising ideas</t>
+          <t>fundraising for soccer teams</t>
         </is>
       </c>
       <c r="G27" s="4" t="n">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="H27" s="5" t="n">
         <v>4</v>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="L27" s="7" t="inlineStr">
         <is>
-          <t>Also covers: track and field fundraiser, cross country fundraising ideas, cross country fundraisers.</t>
+          <t>Also covers: fundraising ideas for soccer clubs.</t>
         </is>
       </c>
     </row>
@@ -2151,16 +2151,16 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Booster Club Fundraising Ideas That Support Every Team in the School</t>
+          <t>Track and Field Fundraising Ideas for Meet Season and Cross Country</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>booster club fundraising ideas</t>
+          <t>track and field fundraising ideas</t>
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>260</v>
+        <v>90</v>
       </c>
       <c r="H28" s="5" t="n">
         <v>4</v>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="L28" s="7" t="inlineStr">
         <is>
-          <t>Also covers: booster club fundraisers, booster fundraising ideas, high school booster club fundraising ideas, athletic booster club fundraising ideas, successful booster clubs.</t>
+          <t>Also covers: track and field fundraiser, cross country fundraising ideas, cross country fundraisers.</t>
         </is>
       </c>
     </row>
@@ -2207,19 +2207,19 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Marching Band Fundraiser Ideas for Competition Season Travel</t>
+          <t>Booster Club Fundraising Ideas That Support Every Team in the School</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>marching band fundraiser ideas</t>
+          <t>booster club fundraising ideas</t>
         </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>90</v>
+        <v>260</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -2234,6 +2234,11 @@
       <c r="K29" t="inlineStr">
         <is>
           <t>Top of funnel</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>Also covers: booster club fundraisers, booster fundraising ideas, high school booster club fundraising ideas, athletic booster club fundraising ideas, successful booster clubs.</t>
         </is>
       </c>
     </row>
@@ -2258,19 +2263,19 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Lacrosse Fundraising Ideas to Pay for Field Time</t>
+          <t>Marching Band Fundraiser Ideas for Competition Season Travel</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>lacrosse fundraising ideas</t>
+          <t>marching band fundraiser ideas</t>
         </is>
       </c>
       <c r="G30" s="4" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -2309,23 +2314,23 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Team Fundraising Ideas for Cheer, Dance, Robotics and Debate Squads</t>
+          <t>Lacrosse Fundraising Ideas to Pay for Field Time</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>team fundraising ideas</t>
+          <t>lacrosse fundraising ideas</t>
         </is>
       </c>
       <c r="G31" s="4" t="n">
-        <v>480</v>
-      </c>
-      <c r="H31" s="9" t="n">
-        <v>18</v>
+        <v>50</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="J31" s="13" t="inlineStr">
@@ -2336,11 +2341,6 @@
       <c r="K31" t="inlineStr">
         <is>
           <t>Top of funnel</t>
-        </is>
-      </c>
-      <c r="L31" s="7" t="inlineStr">
-        <is>
-          <t>Focuses on squads beyond traditional sports; sport-specific ideas have their own articles. Also covers: team fundraisers.</t>
         </is>
       </c>
     </row>
@@ -2365,28 +2365,28 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Fundraiser Ideas for Schools, Teams and Churches, With Setup Time for Each</t>
+          <t>Team Fundraising Ideas for Cheer, Dance, Robotics and Debate Squads</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>fundraiser ideas</t>
+          <t>team fundraising ideas</t>
         </is>
       </c>
       <c r="G32" s="4" t="n">
-        <v>14800</v>
-      </c>
-      <c r="H32" s="11" t="n">
-        <v>36</v>
+        <v>480</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>18</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="J32" s="12" t="inlineStr">
-        <is>
-          <t>School, Church and Club Fundraisers</t>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J32" s="13" t="inlineStr">
+        <is>
+          <t>Fundraisers for Sports Teams</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="L32" s="7" t="inlineStr">
         <is>
-          <t>Also covers: good fundraising ideas, fundraising suggestions, fun fundraiser ideas, fundraising examples.</t>
+          <t>Focuses on squads beyond traditional sports; sport-specific ideas have their own articles. Also covers: team fundraisers.</t>
         </is>
       </c>
     </row>
@@ -2421,19 +2421,19 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Ideas for Schools to Raise Money, Grade by Grade</t>
+          <t>Fundraiser Ideas for Schools, Teams and Churches, With Setup Time for Each</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>ideas for schools to raise money</t>
+          <t>fundraiser ideas</t>
         </is>
       </c>
       <c r="G33" s="4" t="n">
-        <v>5400</v>
+        <v>14800</v>
       </c>
       <c r="H33" s="11" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="L33" s="7" t="inlineStr">
         <is>
-          <t>Also covers: school fundraising ideas, school fundraisers, fundraising opportunities for schools, best school fundraising ideas, unique school fundraising ideas, ways to raise money for schools, easy school fundraisers, how to raise money for school and 1 more.</t>
+          <t>Also covers: good fundraising ideas, fundraising suggestions, fun fundraiser ideas, fundraising examples.</t>
         </is>
       </c>
     </row>
@@ -2477,23 +2477,23 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>School Fundraisers That Make the Most Money per Hour of Work</t>
+          <t>Ideas for Schools to Raise Money, Grade by Grade</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>school fundraisers that make the most money</t>
+          <t>ideas for schools to raise money</t>
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>880</v>
-      </c>
-      <c r="H34" s="9" t="n">
-        <v>29</v>
+        <v>5400</v>
+      </c>
+      <c r="H34" s="11" t="n">
+        <v>31</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="J34" s="12" t="inlineStr">
@@ -2503,12 +2503,12 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="L34" s="7" t="inlineStr">
         <is>
-          <t>Also covers: best school fundraisers, best fundraiser for schools, best fundraisers for elementary schools, what fundraisers bring in the most money, best high school fundraisers.</t>
+          <t>Also covers: school fundraising ideas, school fundraisers, fundraising opportunities for schools, best school fundraising ideas, unique school fundraising ideas, ways to raise money for schools, easy school fundraisers, how to raise money for school and 1 more.</t>
         </is>
       </c>
     </row>
@@ -2533,23 +2533,23 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Winter Fundraising Ideas for January and February</t>
+          <t>School Fundraisers That Make the Most Money per Hour of Work</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>winter fundraising ideas</t>
+          <t>school fundraisers that make the most money</t>
         </is>
       </c>
       <c r="G35" s="4" t="n">
-        <v>260</v>
-      </c>
-      <c r="H35" s="5" t="n">
-        <v>10</v>
+        <v>880</v>
+      </c>
+      <c r="H35" s="9" t="n">
+        <v>29</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Very Easy</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="J35" s="12" t="inlineStr">
@@ -2559,12 +2559,12 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="L35" s="7" t="inlineStr">
         <is>
-          <t>Also covers: winter fundraising ideas schools.</t>
+          <t>Also covers: best school fundraisers, best fundraiser for schools, best fundraisers for elementary schools, what fundraisers bring in the most money, best high school fundraisers.</t>
         </is>
       </c>
     </row>
@@ -39039,7 +39039,7 @@
     <row r="20" ht="75" customHeight="1">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t>Month 1 is the buying layer: the homepage rewrite and the articles closest to a purchase, such as what is in a box, how a World's Finest fundraiser works, and where to buy fundraiser candy bars. Month 2 adds the sports and team articles, the main school, church and nonprofit guides, and seasonal pieces timed for winter and spring. Month 3 completes the school and club articles by grade level and group type, adds youth-group and mission-trip fundraising, and publishes the fall piece early enough to rank before August. Month 1 titles are near-final. Months 2 and 3 are our best current targets based on today's data.</t>
+          <t>Month 1 is the buying layer: the homepage rewrite and the articles closest to a purchase, such as what is in a box, how a World's Finest fundraiser works, and where to buy fundraiser candy bars, plus the Christmas and winter pieces so they rank in time for the season. Month 2 adds the sports and team articles, the main school, church and nonprofit guides, and the spring and Easter pieces, timed to rank before March. Month 3 completes the school and club articles by grade level and group type, adds youth-group and mission-trip fundraising, and publishes the fall piece early enough to rank before August. Month 1 titles are near-final. Months 2 and 3 are our best current targets based on today's data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sotos-produce-market: call-questions slide, no 120 framing
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/sotos-produce-market/keyword-research.xlsx
+++ b/decks/sotos-produce-market/keyword-research.xlsx
@@ -39050,10 +39050,10 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="101" customHeight="1">
+    <row r="23" ht="114" customHeight="1">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>Raw research turned up 1,620 keywords with 529,690 searches a month between them. After removing everything you don't sell or can't serve, 440 keywords with 115,070 searches a month remain, and this plan targets 111,510 of those. That is why the plan has 59 articles instead of our usual 120: going further would have meant near-duplicates or topics that fit you poorly, and the best of those wait on the Bench with the reason for each. Search volumes are national. In the city of Los Angeles, "chocolate fundraiser" gets about 40 searches a month and "fundraiser chocolate bars" about 40, roughly 3% of the US total, and the 14 searches we tested that pair Compton, Long Beach, Carson, Downey, Los Angeles or Southern California with a fundraiser ("compton fundraiser", "chocolate fundraiser los angeles") showed no measurable volume. Visits from farther away build your brand and the chance that AI assistants name your store; walk-in sales come from the local share, your Google listing and the near-me searches the homepage rewrite targets.</t>
+          <t>Raw research turned up 1,620 keywords with 529,690 searches a month between them. After removing everything you don't sell or can't serve, 440 keywords with 115,070 searches a month remain, and this plan targets 111,510 of those. That is why the plan has 59 articles: going further would have meant near-duplicates or topics that fit you poorly. The best of those wait on the Bench with the reason for each, and your answers to the questions below can open up more. Search volumes are national. In the city of Los Angeles, "chocolate fundraiser" gets about 40 searches a month and "fundraiser chocolate bars" about 40, roughly 3% of the US total, and the 14 searches we tested that pair Compton, Long Beach, Carson, Downey, Los Angeles or Southern California with a fundraiser ("compton fundraiser", "chocolate fundraiser los angeles") showed no measurable volume. Visits from farther away build your brand and the chance that AI assistants name your store; walk-in sales come from the local share, your Google listing and the near-me searches the homepage rewrite targets.</t>
         </is>
       </c>
     </row>
@@ -39106,10 +39106,10 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="101" customHeight="1">
+    <row r="35" ht="127" customHeight="1">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>1. Can you claim your Google Business Profile, or is someone else managing it? 2. Is the chocolate counter the part of the business you want to grow online, or should the produce and grocery side get pages too? "Produce market near me" alone gets 6,600 searches a month nationally. 3. Would you like an article in Spanish? Your listing's phone number is your Spanish line, and Spanish chocolate-fundraiser searches come to about 100 a month. 4. Are there nearby cities (Long Beach, Carson, Downey) where groups regularly come from? The searches we tested that pair those cities with a fundraiser showed no measurable volume, so city pages only make sense if that is where your buyers come from. 5. How do organizers find you today: word of mouth, schools, churches, or World's Finest's own store locator? 6. Do you offer anything to groups beyond walk-in boxes, such as holding boxes for a pickup date, and what happens with unsold boxes?</t>
+          <t>1. Can you claim your Google Business Profile, or is someone else managing it? 2. Should your website cover the produce and grocery side? That opens a produce and grocery pillar: "produce market near me" alone gets 6,600 searches a month nationally. 3. Would you like pages in Spanish? That opens a Spanish chocolate-fundraiser article (about 100 searches a month) and Spanish versions of your main pages; your listing's phone is already your Spanish line. 4. Which nearby cities (Long Beach, Carson, Downey) do groups come from? The searches we tested that pair those cities with a fundraiser showed no measurable volume, so city pages only make sense where your buyers come from. 5. Do you carry, or could you carry, other World's Finest products? Mint Meltaways and the 5 lb bar get about 330 searches a month together. 6. What can you offer groups beyond walk-in boxes, such as holding boxes for a pickup date or large orders, and what happens with unsold boxes? Those answers become pages for organizers about to buy. 7. Which groups buy from you the most, and how do they find you today: word of mouth, schools, churches, or World's Finest's own store locator? The answer decides which groups get more articles written for them, and which articles come first.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sotos-produce-market: GBP finding corrected (profile is managed)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/sotos-produce-market/keyword-research.xlsx
+++ b/decks/sotos-produce-market/keyword-research.xlsx
@@ -38716,7 +38716,7 @@
       </c>
       <c r="E3" s="15" t="inlineStr">
         <is>
-          <t>This #1 is your map listing in the local results, not the website. Claiming the listing protects it.</t>
+          <t>This #1 is your map listing in the local results, not the website.</t>
         </is>
       </c>
     </row>
@@ -39008,10 +39008,10 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="49" customHeight="1">
+    <row r="14" ht="75" customHeight="1">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>Your Google Business Profile is the asset that already wins for you, and it is unclaimed. Google Maps lists Soto's Produce Market as a grocery store with 4.4 stars from 312 reviews and shows a "Claim this business" link. Claiming it puts you in control of your hours, photos, website link and review replies. We recommend doing this before anything else in the plan.</t>
+          <t>Your Google Business Profile is the asset that already wins for you. It shows Soto's first in the map results for World's Finest searches near the store and carries 4.4 stars from 312 reviews. Its Insights (calls, direction requests, the searches that found you) are the best measure of your search traffic today, better than anything the website can show yet. Two details need fixing: the listing's phone is your Spanish line while your site leads with (310) 955-3155, and your site's map pin sits half a mile from the listing's. We recommend starting there, together with access to the listing's Insights.</t>
         </is>
       </c>
     </row>
@@ -39109,7 +39109,7 @@
     <row r="35" ht="127" customHeight="1">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>1. Can you claim your Google Business Profile, or is someone else managing it? 2. Should your website cover the produce and grocery side? That opens a produce and grocery pillar: "produce market near me" alone gets 6,600 searches a month nationally. 3. Would you like pages in Spanish? That opens a Spanish chocolate-fundraiser article (about 100 searches a month) and Spanish versions of your main pages; your listing's phone is already your Spanish line. 4. Which nearby cities (Long Beach, Carson, Downey) do groups come from? The searches we tested that pair those cities with a fundraiser showed no measurable volume, so city pages only make sense where your buyers come from. 5. Do you carry, or could you carry, other World's Finest products? Mint Meltaways and the 5 lb bar get about 330 searches a month together. 6. What can you offer groups beyond walk-in boxes, such as holding boxes for a pickup date or large orders, and what happens with unsold boxes? Those answers become pages for organizers about to buy. 7. Which groups buy from you the most, and how do they find you today: word of mouth, schools, churches, or World's Finest's own store locator? The answer decides which groups get more articles written for them, and which articles come first.</t>
+          <t>1. Who manages your Google Business Profile, and can we see its Insights (calls, direction requests, searches)? 2. Should your website cover the produce and grocery side? That opens a produce and grocery pillar: "produce market near me" alone gets 6,600 searches a month nationally. 3. Would you like pages in Spanish? That opens a Spanish chocolate-fundraiser article (about 100 searches a month) and Spanish versions of your main pages; your listing's phone is already your Spanish line. 4. Which nearby cities (Long Beach, Carson, Downey) do groups come from? The searches we tested that pair those cities with a fundraiser showed no measurable volume, so city pages only make sense where your buyers come from. 5. Do you carry, or could you carry, other World's Finest products? Mint Meltaways and the 5 lb bar get about 330 searches a month together. 6. What can you offer groups beyond walk-in boxes, such as holding boxes for a pickup date or large orders, and what happens with unsold boxes? Those answers become pages for organizers about to buy. 7. Which groups buy from you the most, and how do they find you today: word of mouth, schools, churches, or World's Finest's own store locator? The answer decides which groups get more articles written for them, and which articles come first.</t>
         </is>
       </c>
     </row>

</xml_diff>